<commit_message>
updated automation header alignement
</commit_message>
<xml_diff>
--- a/utils/reference/volare_bpi_cards_xdays-header.xlsx
+++ b/utils/reference/volare_bpi_cards_xdays-header.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="11460"/>
+    <workbookView windowWidth="27945" windowHeight="12180"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="77">
   <si>
     <t>CH CODE</t>
   </si>
@@ -56,9 +56,6 @@
     <t>MOBILE_NO</t>
   </si>
   <si>
-    <t>TU</t>
-  </si>
-  <si>
     <t>ADDRESS</t>
   </si>
   <si>
@@ -116,12 +113,6 @@
     <t>LAST DUE DATE</t>
   </si>
   <si>
-    <t>SPOUSE NUMBER</t>
-  </si>
-  <si>
-    <t>TYPE</t>
-  </si>
-  <si>
     <t>Ch Code</t>
   </si>
   <si>
@@ -146,9 +137,6 @@
     <t>mobile_no</t>
   </si>
   <si>
-    <t>tu</t>
-  </si>
-  <si>
     <t>address</t>
   </si>
   <si>
@@ -206,12 +194,6 @@
     <t>last due date</t>
   </si>
   <si>
-    <t>spouse number</t>
-  </si>
-  <si>
-    <t>type</t>
-  </si>
-  <si>
     <t>CUSTOMER ID</t>
   </si>
   <si>
@@ -224,9 +206,6 @@
     <t>HOME_PH</t>
   </si>
   <si>
-    <t>TU_NUMBERS</t>
-  </si>
-  <si>
     <t>PRIMARY ADDRESS</t>
   </si>
   <si>
@@ -258,9 +237,6 @@
   </si>
   <si>
     <t>home_ph</t>
-  </si>
-  <si>
-    <t>tu_numbers</t>
   </si>
   <si>
     <t>primary address</t>
@@ -1449,7 +1425,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AD5"/>
+  <dimension ref="A1:AA5"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
     <col min="2" max="2" width="13.1428571428571" customWidth="1"/>
@@ -1458,31 +1434,28 @@
     <col min="6" max="6" width="10.5714285714286" customWidth="1"/>
     <col min="7" max="7" width="6.57142857142857" customWidth="1"/>
     <col min="8" max="8" width="11.7142857142857" customWidth="1"/>
-    <col min="9" max="9" width="13.1428571428571" customWidth="1"/>
-    <col min="10" max="10" width="17.7142857142857" customWidth="1"/>
-    <col min="11" max="11" width="6.57142857142857" customWidth="1"/>
-    <col min="12" max="12" width="8.28571428571429" customWidth="1"/>
-    <col min="13" max="13" width="18.5714285714286" customWidth="1"/>
-    <col min="14" max="14" width="4.57142857142857" customWidth="1"/>
-    <col min="15" max="15" width="5.42857142857143" customWidth="1"/>
-    <col min="16" max="16" width="6.71428571428571" customWidth="1"/>
-    <col min="17" max="17" width="23.7142857142857" customWidth="1"/>
-    <col min="18" max="18" width="20.8571428571429" customWidth="1"/>
-    <col min="19" max="19" width="21.7142857142857" customWidth="1"/>
-    <col min="20" max="20" width="14.8571428571429" customWidth="1"/>
-    <col min="21" max="21" width="28" customWidth="1"/>
-    <col min="22" max="22" width="11.2857142857143" customWidth="1"/>
-    <col min="23" max="23" width="12.5714285714286" customWidth="1"/>
-    <col min="24" max="24" width="10.7142857142857" customWidth="1"/>
-    <col min="25" max="25" width="12.5714285714286" customWidth="1"/>
-    <col min="26" max="26" width="12" customWidth="1"/>
-    <col min="27" max="27" width="12.8571428571429" customWidth="1"/>
-    <col min="28" max="28" width="14.4285714285714" customWidth="1"/>
-    <col min="29" max="29" width="16.5714285714286" customWidth="1"/>
-    <col min="30" max="30" width="5.28571428571429" customWidth="1"/>
+    <col min="9" max="9" width="17.7142857142857" customWidth="1"/>
+    <col min="10" max="10" width="6.57142857142857" customWidth="1"/>
+    <col min="11" max="11" width="8.28571428571429" customWidth="1"/>
+    <col min="12" max="12" width="18.5714285714286" customWidth="1"/>
+    <col min="13" max="13" width="4.57142857142857" customWidth="1"/>
+    <col min="14" max="14" width="5.42857142857143" customWidth="1"/>
+    <col min="15" max="15" width="6.71428571428571" customWidth="1"/>
+    <col min="16" max="16" width="23.7142857142857" customWidth="1"/>
+    <col min="17" max="17" width="20.8571428571429" customWidth="1"/>
+    <col min="18" max="18" width="21.7142857142857" customWidth="1"/>
+    <col min="19" max="19" width="14.8571428571429" customWidth="1"/>
+    <col min="20" max="20" width="28" customWidth="1"/>
+    <col min="21" max="21" width="11.2857142857143" customWidth="1"/>
+    <col min="22" max="22" width="12.5714285714286" customWidth="1"/>
+    <col min="23" max="23" width="10.7142857142857" customWidth="1"/>
+    <col min="24" max="24" width="12.5714285714286" customWidth="1"/>
+    <col min="25" max="25" width="12" customWidth="1"/>
+    <col min="26" max="26" width="12.8571428571429" customWidth="1"/>
+    <col min="27" max="27" width="14.4285714285714" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30">
+    <row r="1" spans="1:27">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1564,114 +1537,96 @@
       <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:27">
+      <c r="A2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>29</v>
       </c>
+      <c r="D2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="Z2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>53</v>
+      </c>
     </row>
-    <row r="2" spans="1:30">
-      <c r="A2" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="R2" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="S2" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="T2" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="U2" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="V2" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="W2" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="X2" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="Y2" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="Z2" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="AA2" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="AB2" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="AC2" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="AD2" s="2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="3" spans="1:27">
+    <row r="3" spans="1:26">
       <c r="A3" t="s">
         <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="C3" t="s">
         <v>2</v>
@@ -1680,58 +1635,58 @@
         <v>3</v>
       </c>
       <c r="E3" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="F3" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="G3" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="H3" t="s">
         <v>7</v>
       </c>
       <c r="I3" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="J3" t="s">
-        <v>65</v>
+        <v>9</v>
       </c>
       <c r="K3" t="s">
         <v>10</v>
       </c>
       <c r="L3" t="s">
-        <v>11</v>
+        <v>59</v>
       </c>
       <c r="M3" t="s">
-        <v>66</v>
+        <v>12</v>
       </c>
       <c r="N3" t="s">
         <v>13</v>
       </c>
       <c r="O3" t="s">
-        <v>14</v>
+        <v>60</v>
       </c>
       <c r="P3" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="Q3" t="s">
-        <v>68</v>
+        <v>16</v>
       </c>
       <c r="R3" t="s">
-        <v>17</v>
+        <v>62</v>
       </c>
       <c r="S3" t="s">
-        <v>69</v>
-      </c>
-      <c r="T3" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="U3" t="s">
+        <v>63</v>
       </c>
       <c r="V3" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="W3" t="s">
-        <v>71</v>
+        <v>22</v>
       </c>
       <c r="X3" t="s">
         <v>23</v>
@@ -1742,93 +1697,87 @@
       <c r="Z3" t="s">
         <v>25</v>
       </c>
-      <c r="AA3" t="s">
-        <v>26</v>
-      </c>
     </row>
-    <row r="4" spans="1:27">
+    <row r="4" spans="1:26">
       <c r="A4" t="s">
         <v>0</v>
       </c>
       <c r="B4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" t="s">
+        <v>66</v>
+      </c>
+      <c r="F4" t="s">
+        <v>67</v>
+      </c>
+      <c r="G4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" t="s">
+        <v>69</v>
+      </c>
+      <c r="J4" t="s">
+        <v>36</v>
+      </c>
+      <c r="K4" t="s">
+        <v>37</v>
+      </c>
+      <c r="L4" t="s">
+        <v>70</v>
+      </c>
+      <c r="M4" t="s">
+        <v>39</v>
+      </c>
+      <c r="N4" t="s">
+        <v>40</v>
+      </c>
+      <c r="O4" t="s">
+        <v>71</v>
+      </c>
+      <c r="P4" t="s">
         <v>72</v>
       </c>
-      <c r="C4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D4" t="s">
-        <v>33</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="Q4" t="s">
+        <v>43</v>
+      </c>
+      <c r="R4" t="s">
         <v>73</v>
       </c>
-      <c r="F4" t="s">
+      <c r="S4" t="s">
+        <v>45</v>
+      </c>
+      <c r="U4" t="s">
         <v>74</v>
       </c>
-      <c r="G4" t="s">
+      <c r="V4" t="s">
         <v>75</v>
       </c>
-      <c r="H4" t="s">
-        <v>37</v>
-      </c>
-      <c r="I4" t="s">
+      <c r="W4" t="s">
+        <v>49</v>
+      </c>
+      <c r="X4" t="s">
+        <v>50</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="17:17">
+      <c r="Q5" t="s">
         <v>76</v>
-      </c>
-      <c r="J4" t="s">
-        <v>77</v>
-      </c>
-      <c r="K4" t="s">
-        <v>40</v>
-      </c>
-      <c r="L4" t="s">
-        <v>41</v>
-      </c>
-      <c r="M4" t="s">
-        <v>78</v>
-      </c>
-      <c r="N4" t="s">
-        <v>43</v>
-      </c>
-      <c r="O4" t="s">
-        <v>44</v>
-      </c>
-      <c r="P4" t="s">
-        <v>79</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>80</v>
-      </c>
-      <c r="R4" t="s">
-        <v>47</v>
-      </c>
-      <c r="S4" t="s">
-        <v>81</v>
-      </c>
-      <c r="T4" t="s">
-        <v>49</v>
-      </c>
-      <c r="V4" t="s">
-        <v>82</v>
-      </c>
-      <c r="W4" t="s">
-        <v>83</v>
-      </c>
-      <c r="X4" t="s">
-        <v>53</v>
-      </c>
-      <c r="Y4" t="s">
-        <v>54</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>55</v>
-      </c>
-      <c r="AA4" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="5" spans="18:18">
-      <c r="R5" t="s">
-        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>